<commit_message>
update my daily log
</commit_message>
<xml_diff>
--- a/1234567.xlsx
+++ b/1234567.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5731650e8b717ef2/Desktop/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="132" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{497D8C1F-8550-4D6A-82FB-21A58DF8F71D}"/>
+  <xr:revisionPtr revIDLastSave="146" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3DA88CF-A283-4040-9D55-5EAE3A7696A8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t>Done good questions on recursion</t>
+  </si>
+  <si>
+    <t>I have done a lot of problems on python which increased my confidence</t>
   </si>
 </sst>
 </file>
@@ -1439,27 +1442,51 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A15" s="12"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="14" t="str">
+    <row r="15" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="12">
+        <v>46278</v>
+      </c>
+      <c r="B15" s="13">
+        <v>360</v>
+      </c>
+      <c r="C15" s="13">
+        <v>60</v>
+      </c>
+      <c r="D15" s="13">
+        <v>300</v>
+      </c>
+      <c r="E15" s="13">
+        <v>180</v>
+      </c>
+      <c r="F15" s="13">
+        <v>0</v>
+      </c>
+      <c r="G15" s="13">
+        <v>0</v>
+      </c>
+      <c r="H15" s="13">
+        <v>240</v>
+      </c>
+      <c r="I15" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="14" t="str">
+        <v>1140</v>
+      </c>
+      <c r="J15" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
-      <c r="N15" s="16"/>
+        <v>300</v>
+      </c>
+      <c r="K15" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="L15" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="M15" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="N15" s="16" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="12"/>

</xml_diff>